<commit_message>
keyword for tablet and liquids modified
</commit_message>
<xml_diff>
--- a/inst/extdata/medicaton_costs_all.xlsx
+++ b/inst/extdata/medicaton_costs_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sheej\Documents\Sheeja_WinLap\repos\packDAMipd\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D31BC17C-1180-49AB-B822-8CF32AF217B0}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4F4F3D9-2476-4853-BFBE-90FB610EF142}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$407</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1164,7 +1163,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:J407"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1210,7 +1208,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="2" spans="1:10" ht="22.5" customHeight="1">
       <c r="A2" s="8" t="s">
         <v>8</v>
       </c>
@@ -1241,7 +1239,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="3" spans="1:10" ht="22.5" customHeight="1">
       <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
@@ -1272,7 +1270,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="4" spans="1:10" ht="22.5" customHeight="1">
       <c r="A4" s="8" t="s">
         <v>8</v>
       </c>
@@ -1303,7 +1301,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="5" spans="1:10" ht="22.5" customHeight="1">
       <c r="A5" s="8" t="s">
         <v>8</v>
       </c>
@@ -1334,7 +1332,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="6" spans="1:10" ht="22.5" customHeight="1">
       <c r="A6" s="8" t="s">
         <v>8</v>
       </c>
@@ -1365,7 +1363,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="7" spans="1:10" ht="22.5" customHeight="1">
       <c r="A7" s="8" t="s">
         <v>8</v>
       </c>
@@ -1396,7 +1394,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="8" spans="1:10" ht="22.5" customHeight="1">
       <c r="A8" s="8" t="s">
         <v>15</v>
       </c>
@@ -1429,7 +1427,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="9" spans="1:10" ht="22.5" customHeight="1">
       <c r="A9" s="8" t="s">
         <v>20</v>
       </c>
@@ -1462,7 +1460,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="10" spans="1:10" ht="22.5" customHeight="1">
       <c r="A10" s="8" t="s">
         <v>23</v>
       </c>
@@ -1495,7 +1493,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="11" spans="1:10" ht="22.5" customHeight="1">
       <c r="A11" s="8" t="s">
         <v>27</v>
       </c>
@@ -1528,7 +1526,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="12" spans="1:10" ht="22.5" customHeight="1">
       <c r="A12" s="8" t="s">
         <v>27</v>
       </c>
@@ -1561,7 +1559,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="13" spans="1:10" ht="22.5" customHeight="1">
       <c r="A13" s="8" t="s">
         <v>27</v>
       </c>
@@ -1594,7 +1592,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="14" spans="1:10" ht="22.5" customHeight="1">
       <c r="A14" s="8" t="s">
         <v>32</v>
       </c>
@@ -1627,7 +1625,7 @@
         <v>per Vial</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="15" spans="1:10" ht="22.5" customHeight="1">
       <c r="A15" s="8" t="s">
         <v>35</v>
       </c>
@@ -1660,7 +1658,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="16" spans="1:10" ht="22.5" customHeight="1">
       <c r="A16" s="8" t="s">
         <v>39</v>
       </c>
@@ -1693,7 +1691,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="17" spans="1:10" ht="22.5" customHeight="1">
       <c r="A17" s="8" t="s">
         <v>39</v>
       </c>
@@ -1726,7 +1724,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="18" spans="1:10" ht="22.5" customHeight="1">
       <c r="A18" s="8" t="s">
         <v>39</v>
       </c>
@@ -1759,7 +1757,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="19" spans="1:10" ht="22.5" customHeight="1">
       <c r="A19" s="8" t="s">
         <v>39</v>
       </c>
@@ -1792,7 +1790,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="20" spans="1:10" ht="22.5" customHeight="1">
       <c r="A20" s="8" t="s">
         <v>39</v>
       </c>
@@ -1825,7 +1823,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="21" spans="1:10" ht="22.5" customHeight="1">
       <c r="A21" s="8" t="s">
         <v>39</v>
       </c>
@@ -1858,7 +1856,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="22" spans="1:10" ht="22.5" customHeight="1">
       <c r="A22" s="8" t="s">
         <v>39</v>
       </c>
@@ -1891,7 +1889,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="23" spans="1:10" ht="22.5" customHeight="1">
       <c r="A23" s="8" t="s">
         <v>39</v>
       </c>
@@ -1924,7 +1922,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="24" spans="1:10" ht="22.5" customHeight="1">
       <c r="A24" s="8" t="s">
         <v>39</v>
       </c>
@@ -1957,7 +1955,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="25" spans="1:10" ht="22.5" customHeight="1">
       <c r="A25" s="8" t="s">
         <v>50</v>
       </c>
@@ -1990,7 +1988,7 @@
         <v>per Vial</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="26" spans="1:10" ht="22.5" customHeight="1">
       <c r="A26" s="8" t="s">
         <v>50</v>
       </c>
@@ -2023,7 +2021,7 @@
         <v>per Vial</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="27" spans="1:10" ht="22.5" customHeight="1">
       <c r="A27" s="8" t="s">
         <v>50</v>
       </c>
@@ -2056,7 +2054,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="28" spans="1:10" ht="22.5" customHeight="1">
       <c r="A28" s="8" t="s">
         <v>50</v>
       </c>
@@ -2089,7 +2087,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="29" spans="1:10" ht="22.5" customHeight="1">
       <c r="A29" s="8" t="s">
         <v>50</v>
       </c>
@@ -2122,7 +2120,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="30" spans="1:10" ht="22.5" customHeight="1">
       <c r="A30" s="8" t="s">
         <v>50</v>
       </c>
@@ -2155,7 +2153,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="31" spans="1:10" ht="22.5" customHeight="1">
       <c r="A31" s="8" t="s">
         <v>50</v>
       </c>
@@ -2188,7 +2186,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="32" spans="1:10" ht="22.5" customHeight="1">
       <c r="A32" s="8" t="s">
         <v>50</v>
       </c>
@@ -2221,7 +2219,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="33" spans="1:10" ht="22.5" customHeight="1">
       <c r="A33" s="8" t="s">
         <v>50</v>
       </c>
@@ -2254,7 +2252,7 @@
         <v>per Vial</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="34" spans="1:10" ht="22.5" customHeight="1">
       <c r="A34" s="8" t="s">
         <v>50</v>
       </c>
@@ -2287,7 +2285,7 @@
         <v>per Vial</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="35" spans="1:10" ht="22.5" customHeight="1">
       <c r="A35" s="8" t="s">
         <v>50</v>
       </c>
@@ -2320,7 +2318,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="36" spans="1:10" ht="22.5" customHeight="1">
       <c r="A36" s="8" t="s">
         <v>50</v>
       </c>
@@ -2353,7 +2351,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="37" spans="1:10" ht="22.5" customHeight="1">
       <c r="A37" s="8" t="s">
         <v>66</v>
       </c>
@@ -2386,7 +2384,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="38" spans="1:10" ht="22.5" customHeight="1">
       <c r="A38" s="8" t="s">
         <v>66</v>
       </c>
@@ -2419,7 +2417,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="39" spans="1:10" ht="22.5" customHeight="1">
       <c r="A39" s="8" t="s">
         <v>66</v>
       </c>
@@ -2452,7 +2450,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="40" spans="1:10" ht="22.5" customHeight="1">
       <c r="A40" s="8" t="s">
         <v>66</v>
       </c>
@@ -2485,7 +2483,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="41" spans="1:10" ht="22.5" customHeight="1">
       <c r="A41" s="8" t="s">
         <v>66</v>
       </c>
@@ -2518,7 +2516,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="42" spans="1:10" ht="22.5" customHeight="1">
       <c r="A42" s="8" t="s">
         <v>66</v>
       </c>
@@ -2551,7 +2549,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="43" spans="1:10" ht="22.5" customHeight="1">
       <c r="A43" s="8" t="s">
         <v>66</v>
       </c>
@@ -2584,7 +2582,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="44" spans="1:10" ht="22.5" customHeight="1">
       <c r="A44" s="8" t="s">
         <v>66</v>
       </c>
@@ -2617,7 +2615,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="45" spans="1:10" ht="22.5" customHeight="1">
       <c r="A45" s="8" t="s">
         <v>66</v>
       </c>
@@ -2650,7 +2648,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="46" spans="1:10" ht="22.5" customHeight="1">
       <c r="A46" s="8" t="s">
         <v>66</v>
       </c>
@@ -2683,7 +2681,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="47" spans="1:10" ht="22.5" customHeight="1">
       <c r="A47" s="8" t="s">
         <v>66</v>
       </c>
@@ -2716,7 +2714,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="48" spans="1:10" ht="22.5" customHeight="1">
       <c r="A48" s="8" t="s">
         <v>66</v>
       </c>
@@ -2749,7 +2747,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="49" spans="1:10" ht="22.5" customHeight="1">
       <c r="A49" s="8" t="s">
         <v>69</v>
       </c>
@@ -2782,7 +2780,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="50" spans="1:10" ht="22.5" customHeight="1">
       <c r="A50" s="8" t="s">
         <v>69</v>
       </c>
@@ -2815,7 +2813,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="51" spans="1:10" ht="22.5" customHeight="1">
       <c r="A51" s="8" t="s">
         <v>69</v>
       </c>
@@ -2848,7 +2846,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="52" spans="1:10" ht="22.5" customHeight="1">
       <c r="A52" s="8" t="s">
         <v>71</v>
       </c>
@@ -2881,7 +2879,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="53" spans="1:10" ht="22.5" customHeight="1">
       <c r="A53" s="8" t="s">
         <v>71</v>
       </c>
@@ -2914,7 +2912,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="54" spans="1:10" ht="22.5" customHeight="1">
       <c r="A54" s="8" t="s">
         <v>71</v>
       </c>
@@ -2947,7 +2945,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="55" spans="1:10" ht="22.5" customHeight="1">
       <c r="A55" s="8" t="s">
         <v>71</v>
       </c>
@@ -2980,7 +2978,7 @@
         <v>per Ampoule</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="56" spans="1:10" ht="22.5" customHeight="1">
       <c r="A56" s="8" t="s">
         <v>20</v>
       </c>
@@ -3013,7 +3011,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="57" spans="1:10" ht="22.5" customHeight="1">
       <c r="A57" s="8" t="s">
         <v>20</v>
       </c>
@@ -3046,7 +3044,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="58" spans="1:10" ht="22.5" customHeight="1">
       <c r="A58" s="8" t="s">
         <v>20</v>
       </c>
@@ -3079,7 +3077,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="59" spans="1:10" ht="22.5" customHeight="1">
       <c r="A59" s="8" t="s">
         <v>20</v>
       </c>
@@ -3112,7 +3110,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="60" spans="1:10" ht="22.5" customHeight="1">
       <c r="A60" s="8" t="s">
         <v>20</v>
       </c>
@@ -3145,7 +3143,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="61" spans="1:10" ht="22.5" customHeight="1">
       <c r="A61" s="8" t="s">
         <v>23</v>
       </c>
@@ -3178,7 +3176,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="62" spans="1:10" ht="22.5" customHeight="1">
       <c r="A62" s="8" t="s">
         <v>82</v>
       </c>
@@ -3211,7 +3209,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="63" spans="1:10" ht="22.5" customHeight="1">
       <c r="A63" s="8" t="s">
         <v>82</v>
       </c>
@@ -3244,7 +3242,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="64" spans="1:10" ht="22.5" customHeight="1">
       <c r="A64" s="8" t="s">
         <v>82</v>
       </c>
@@ -3277,7 +3275,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="65" spans="1:10" ht="22.5" customHeight="1">
       <c r="A65" s="8" t="s">
         <v>82</v>
       </c>
@@ -3310,7 +3308,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="66" spans="1:10" ht="22.5" customHeight="1">
       <c r="A66" s="8" t="s">
         <v>82</v>
       </c>
@@ -3343,7 +3341,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="67" spans="1:10" ht="22.5" customHeight="1">
       <c r="A67" s="8" t="s">
         <v>82</v>
       </c>
@@ -3376,7 +3374,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="68" spans="1:10" ht="22.5" customHeight="1">
       <c r="A68" s="8" t="s">
         <v>82</v>
       </c>
@@ -3409,7 +3407,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="69" spans="1:10" ht="22.5" customHeight="1">
       <c r="A69" s="8" t="s">
         <v>82</v>
       </c>
@@ -3442,7 +3440,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="70" spans="1:10" ht="22.5" customHeight="1">
       <c r="A70" s="8" t="s">
         <v>82</v>
       </c>
@@ -3475,7 +3473,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="71" spans="1:10" ht="22.5" customHeight="1">
       <c r="A71" s="8" t="s">
         <v>82</v>
       </c>
@@ -3508,7 +3506,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="72" spans="1:10" ht="22.5" customHeight="1">
       <c r="A72" s="8" t="s">
         <v>82</v>
       </c>
@@ -3541,7 +3539,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="73" spans="1:10" ht="22.5" customHeight="1">
       <c r="A73" s="8" t="s">
         <v>82</v>
       </c>
@@ -3574,7 +3572,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="74" spans="1:10" ht="22.5" customHeight="1">
       <c r="A74" s="8" t="s">
         <v>82</v>
       </c>
@@ -3607,7 +3605,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="75" spans="1:10" ht="22.5" customHeight="1">
       <c r="A75" s="8" t="s">
         <v>82</v>
       </c>
@@ -3640,7 +3638,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="76" spans="1:10" ht="22.5" customHeight="1">
       <c r="A76" s="8" t="s">
         <v>82</v>
       </c>
@@ -3673,7 +3671,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="77" spans="1:10" ht="22.5" customHeight="1">
       <c r="A77" s="8" t="s">
         <v>82</v>
       </c>
@@ -3706,7 +3704,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="78" spans="1:10" ht="22.5" customHeight="1">
       <c r="A78" s="8" t="s">
         <v>50</v>
       </c>
@@ -3739,7 +3737,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="79" spans="1:10" ht="22.5" customHeight="1">
       <c r="A79" s="8" t="s">
         <v>50</v>
       </c>
@@ -3772,7 +3770,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="80" spans="1:10" ht="22.5" customHeight="1">
       <c r="A80" s="8" t="s">
         <v>50</v>
       </c>
@@ -3805,7 +3803,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="81" spans="1:10" ht="22.5" customHeight="1">
       <c r="A81" s="8" t="s">
         <v>50</v>
       </c>
@@ -3838,7 +3836,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="82" spans="1:10" ht="22.5" customHeight="1">
       <c r="A82" s="8" t="s">
         <v>50</v>
       </c>
@@ -3871,7 +3869,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="83" spans="1:10" ht="22.5" customHeight="1">
       <c r="A83" s="8" t="s">
         <v>50</v>
       </c>
@@ -3904,7 +3902,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="84" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="84" spans="1:10" ht="22.5" customHeight="1">
       <c r="A84" s="8" t="s">
         <v>50</v>
       </c>
@@ -3937,7 +3935,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="85" spans="1:10" ht="22.5" customHeight="1">
       <c r="A85" s="8" t="s">
         <v>50</v>
       </c>
@@ -3970,7 +3968,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="86" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="86" spans="1:10" ht="22.5" customHeight="1">
       <c r="A86" s="8" t="s">
         <v>66</v>
       </c>
@@ -4003,7 +4001,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="87" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="87" spans="1:10" ht="22.5" customHeight="1">
       <c r="A87" s="8" t="s">
         <v>66</v>
       </c>
@@ -4036,7 +4034,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="88" spans="1:10" ht="22.5" customHeight="1">
       <c r="A88" s="8" t="s">
         <v>66</v>
       </c>
@@ -4069,7 +4067,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="89" spans="1:10" ht="22.5" customHeight="1">
       <c r="A89" s="8" t="s">
         <v>66</v>
       </c>
@@ -4102,7 +4100,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="90" spans="1:10" ht="22.5" customHeight="1">
       <c r="A90" s="8" t="s">
         <v>66</v>
       </c>
@@ -4135,7 +4133,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="91" spans="1:10" ht="22.5" customHeight="1">
       <c r="A91" s="8" t="s">
         <v>66</v>
       </c>
@@ -4168,7 +4166,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="92" spans="1:10" ht="22.5" customHeight="1">
       <c r="A92" s="8" t="s">
         <v>88</v>
       </c>
@@ -4201,7 +4199,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="93" spans="1:10" ht="22.5" customHeight="1">
       <c r="A93" s="8" t="s">
         <v>88</v>
       </c>
@@ -4234,7 +4232,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="94" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="94" spans="1:10" ht="22.5" customHeight="1">
       <c r="A94" s="8" t="s">
         <v>71</v>
       </c>
@@ -4267,7 +4265,7 @@
         <v>per Bottle</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="95" spans="1:10" ht="22.5" customHeight="1">
       <c r="A95" s="8" t="s">
         <v>15</v>
       </c>
@@ -4298,7 +4296,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="96" spans="1:10" ht="22.5" customHeight="1">
       <c r="A96" s="8" t="s">
         <v>15</v>
       </c>
@@ -4329,7 +4327,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="97" spans="1:10" ht="22.5" customHeight="1">
       <c r="A97" s="8" t="s">
         <v>15</v>
       </c>
@@ -4360,7 +4358,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="98" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="98" spans="1:10" ht="22.5" customHeight="1">
       <c r="A98" s="8" t="s">
         <v>15</v>
       </c>
@@ -4391,7 +4389,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="99" spans="1:10" ht="22.5" customHeight="1">
       <c r="A99" s="8" t="s">
         <v>15</v>
       </c>
@@ -4422,7 +4420,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="100" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="100" spans="1:10" ht="22.5" customHeight="1">
       <c r="A100" s="8" t="s">
         <v>15</v>
       </c>
@@ -4453,7 +4451,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="101" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="101" spans="1:10" ht="22.5" customHeight="1">
       <c r="A101" s="8" t="s">
         <v>15</v>
       </c>
@@ -4484,7 +4482,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="102" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="102" spans="1:10" ht="22.5" customHeight="1">
       <c r="A102" s="8" t="s">
         <v>15</v>
       </c>
@@ -4515,7 +4513,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="103" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="103" spans="1:10" ht="22.5" customHeight="1">
       <c r="A103" s="8" t="s">
         <v>15</v>
       </c>
@@ -4546,7 +4544,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="104" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="104" spans="1:10" ht="22.5" customHeight="1">
       <c r="A104" s="8" t="s">
         <v>15</v>
       </c>
@@ -4577,7 +4575,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="105" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="105" spans="1:10" ht="22.5" customHeight="1">
       <c r="A105" s="8" t="s">
         <v>15</v>
       </c>
@@ -4608,7 +4606,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="106" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="106" spans="1:10" ht="22.5" customHeight="1">
       <c r="A106" s="8" t="s">
         <v>15</v>
       </c>
@@ -4639,7 +4637,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="107" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="107" spans="1:10" ht="22.5" customHeight="1">
       <c r="A107" s="8" t="s">
         <v>15</v>
       </c>
@@ -4670,7 +4668,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="108" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="108" spans="1:10" ht="22.5" customHeight="1">
       <c r="A108" s="8" t="s">
         <v>15</v>
       </c>
@@ -4701,7 +4699,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="109" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="109" spans="1:10" ht="22.5" customHeight="1">
       <c r="A109" s="8" t="s">
         <v>15</v>
       </c>
@@ -4732,7 +4730,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="110" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="110" spans="1:10" ht="22.5" customHeight="1">
       <c r="A110" s="8" t="s">
         <v>15</v>
       </c>
@@ -4763,7 +4761,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="111" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="111" spans="1:10" ht="22.5" customHeight="1">
       <c r="A111" s="8" t="s">
         <v>15</v>
       </c>
@@ -4794,7 +4792,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="112" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="112" spans="1:10" ht="22.5" customHeight="1">
       <c r="A112" s="8" t="s">
         <v>15</v>
       </c>
@@ -4825,7 +4823,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="113" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="113" spans="1:10" ht="22.5" customHeight="1">
       <c r="A113" s="8" t="s">
         <v>15</v>
       </c>
@@ -4856,7 +4854,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="114" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="114" spans="1:10" ht="22.5" customHeight="1">
       <c r="A114" s="8" t="s">
         <v>15</v>
       </c>
@@ -4887,7 +4885,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="115" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="115" spans="1:10" ht="22.5" customHeight="1">
       <c r="A115" s="8" t="s">
         <v>15</v>
       </c>
@@ -4918,7 +4916,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="116" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="116" spans="1:10" ht="22.5" customHeight="1">
       <c r="A116" s="8" t="s">
         <v>15</v>
       </c>
@@ -4949,7 +4947,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="117" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="117" spans="1:10" ht="22.5" customHeight="1">
       <c r="A117" s="8" t="s">
         <v>15</v>
       </c>
@@ -4980,7 +4978,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="118" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="118" spans="1:10" ht="22.5" customHeight="1">
       <c r="A118" s="8" t="s">
         <v>15</v>
       </c>
@@ -5011,7 +5009,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="119" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="119" spans="1:10" ht="22.5" customHeight="1">
       <c r="A119" s="8" t="s">
         <v>15</v>
       </c>
@@ -5042,7 +5040,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="120" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="120" spans="1:10" ht="22.5" customHeight="1">
       <c r="A120" s="8" t="s">
         <v>15</v>
       </c>
@@ -5073,7 +5071,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="121" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="121" spans="1:10" ht="22.5" customHeight="1">
       <c r="A121" s="8" t="s">
         <v>15</v>
       </c>
@@ -5104,7 +5102,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="122" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="122" spans="1:10" ht="22.5" customHeight="1">
       <c r="A122" s="8" t="s">
         <v>15</v>
       </c>
@@ -5135,7 +5133,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="123" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="123" spans="1:10" ht="22.5" customHeight="1">
       <c r="A123" s="8" t="s">
         <v>15</v>
       </c>
@@ -5166,7 +5164,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="124" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="124" spans="1:10" ht="22.5" customHeight="1">
       <c r="A124" s="8" t="s">
         <v>15</v>
       </c>
@@ -5197,7 +5195,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="125" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="125" spans="1:10" ht="22.5" customHeight="1">
       <c r="A125" s="8" t="s">
         <v>15</v>
       </c>
@@ -5228,7 +5226,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="126" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="126" spans="1:10" ht="22.5" customHeight="1">
       <c r="A126" s="8" t="s">
         <v>15</v>
       </c>
@@ -5259,7 +5257,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="127" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="127" spans="1:10" ht="22.5" customHeight="1">
       <c r="A127" s="8" t="s">
         <v>15</v>
       </c>
@@ -5290,7 +5288,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="128" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="128" spans="1:10" ht="22.5" customHeight="1">
       <c r="A128" s="8" t="s">
         <v>15</v>
       </c>
@@ -5321,7 +5319,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="129" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="129" spans="1:10" ht="22.5" customHeight="1">
       <c r="A129" s="8" t="s">
         <v>15</v>
       </c>
@@ -5352,7 +5350,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="130" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="130" spans="1:10" ht="22.5" customHeight="1">
       <c r="A130" s="8" t="s">
         <v>15</v>
       </c>
@@ -5383,7 +5381,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="131" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="131" spans="1:10" ht="22.5" customHeight="1">
       <c r="A131" s="8" t="s">
         <v>27</v>
       </c>
@@ -5414,7 +5412,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="132" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="132" spans="1:10" ht="22.5" customHeight="1">
       <c r="A132" s="8" t="s">
         <v>27</v>
       </c>
@@ -5445,7 +5443,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="133" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="133" spans="1:10" ht="22.5" customHeight="1">
       <c r="A133" s="8" t="s">
         <v>27</v>
       </c>
@@ -5476,7 +5474,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="134" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="134" spans="1:10" ht="22.5" customHeight="1">
       <c r="A134" s="8" t="s">
         <v>27</v>
       </c>
@@ -5507,7 +5505,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="135" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="135" spans="1:10" ht="22.5" customHeight="1">
       <c r="A135" s="8" t="s">
         <v>27</v>
       </c>
@@ -5538,7 +5536,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="136" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="136" spans="1:10" ht="22.5" customHeight="1">
       <c r="A136" s="8" t="s">
         <v>27</v>
       </c>
@@ -5569,7 +5567,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="137" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="137" spans="1:10" ht="22.5" customHeight="1">
       <c r="A137" s="8" t="s">
         <v>27</v>
       </c>
@@ -5598,7 +5596,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="138" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="138" spans="1:10" ht="22.5" customHeight="1">
       <c r="A138" s="8" t="s">
         <v>27</v>
       </c>
@@ -5627,7 +5625,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="139" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="139" spans="1:10" ht="22.5" customHeight="1">
       <c r="A139" s="8" t="s">
         <v>27</v>
       </c>
@@ -5658,7 +5656,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="140" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="140" spans="1:10" ht="22.5" customHeight="1">
       <c r="A140" s="8" t="s">
         <v>27</v>
       </c>
@@ -5689,7 +5687,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="141" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="141" spans="1:10" ht="22.5" customHeight="1">
       <c r="A141" s="8" t="s">
         <v>27</v>
       </c>
@@ -5720,7 +5718,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="142" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="142" spans="1:10" ht="22.5" customHeight="1">
       <c r="A142" s="8" t="s">
         <v>27</v>
       </c>
@@ -5751,7 +5749,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="143" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="143" spans="1:10" ht="22.5" customHeight="1">
       <c r="A143" s="8" t="s">
         <v>27</v>
       </c>
@@ -5782,7 +5780,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="144" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="144" spans="1:10" ht="22.5" customHeight="1">
       <c r="A144" s="8" t="s">
         <v>27</v>
       </c>
@@ -5813,7 +5811,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="145" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="145" spans="1:10" ht="22.5" customHeight="1">
       <c r="A145" s="8" t="s">
         <v>27</v>
       </c>
@@ -5844,7 +5842,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="146" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="146" spans="1:10" ht="22.5" customHeight="1">
       <c r="A146" s="8" t="s">
         <v>27</v>
       </c>
@@ -5873,7 +5871,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="147" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="147" spans="1:10" ht="22.5" customHeight="1">
       <c r="A147" s="8" t="s">
         <v>27</v>
       </c>
@@ -5902,7 +5900,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="148" spans="1:10" ht="22.5" customHeight="1">
       <c r="A148" s="8" t="s">
         <v>27</v>
       </c>
@@ -5933,7 +5931,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="149" spans="1:10" ht="22.5" customHeight="1">
       <c r="A149" s="8" t="s">
         <v>27</v>
       </c>
@@ -5964,7 +5962,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="150" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="150" spans="1:10" ht="22.5" customHeight="1">
       <c r="A150" s="8" t="s">
         <v>27</v>
       </c>
@@ -5995,7 +5993,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="151" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="151" spans="1:10" ht="22.5" customHeight="1">
       <c r="A151" s="8" t="s">
         <v>27</v>
       </c>
@@ -6026,7 +6024,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="152" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="152" spans="1:10" ht="22.5" customHeight="1">
       <c r="A152" s="8" t="s">
         <v>27</v>
       </c>
@@ -6057,7 +6055,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="153" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="153" spans="1:10" ht="22.5" customHeight="1">
       <c r="A153" s="8" t="s">
         <v>27</v>
       </c>
@@ -6088,7 +6086,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="154" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="154" spans="1:10" ht="22.5" customHeight="1">
       <c r="A154" s="8" t="s">
         <v>27</v>
       </c>
@@ -6119,7 +6117,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="155" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="155" spans="1:10" ht="22.5" customHeight="1">
       <c r="A155" s="8" t="s">
         <v>27</v>
       </c>
@@ -6148,7 +6146,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="156" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="156" spans="1:10" ht="22.5" customHeight="1">
       <c r="A156" s="8" t="s">
         <v>27</v>
       </c>
@@ -6177,7 +6175,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="157" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="157" spans="1:10" ht="22.5" customHeight="1">
       <c r="A157" s="8" t="s">
         <v>27</v>
       </c>
@@ -6206,7 +6204,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="158" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="158" spans="1:10" ht="22.5" customHeight="1">
       <c r="A158" s="8" t="s">
         <v>27</v>
       </c>
@@ -6237,7 +6235,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="159" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="159" spans="1:10" ht="22.5" customHeight="1">
       <c r="A159" s="8" t="s">
         <v>27</v>
       </c>
@@ -6268,7 +6266,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="160" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="160" spans="1:10" ht="22.5" customHeight="1">
       <c r="A160" s="8" t="s">
         <v>27</v>
       </c>
@@ -6299,7 +6297,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="161" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="161" spans="1:10" ht="22.5" customHeight="1">
       <c r="A161" s="8" t="s">
         <v>27</v>
       </c>
@@ -6330,7 +6328,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="162" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="162" spans="1:10" ht="22.5" customHeight="1">
       <c r="A162" s="8" t="s">
         <v>27</v>
       </c>
@@ -6361,7 +6359,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="163" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="163" spans="1:10" ht="22.5" customHeight="1">
       <c r="A163" s="8" t="s">
         <v>27</v>
       </c>
@@ -6392,7 +6390,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="164" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="164" spans="1:10" ht="22.5" customHeight="1">
       <c r="A164" s="8" t="s">
         <v>27</v>
       </c>
@@ -6421,7 +6419,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="165" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="165" spans="1:10" ht="22.5" customHeight="1">
       <c r="A165" s="8" t="s">
         <v>27</v>
       </c>
@@ -6450,7 +6448,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="166" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="166" spans="1:10" ht="22.5" customHeight="1">
       <c r="A166" s="8" t="s">
         <v>27</v>
       </c>
@@ -6479,7 +6477,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="167" spans="1:10" ht="39" hidden="1" customHeight="1">
+    <row r="167" spans="1:10" ht="39" customHeight="1">
       <c r="A167" s="8" t="s">
         <v>27</v>
       </c>
@@ -6510,7 +6508,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="168" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="168" spans="1:10" ht="22.5" customHeight="1">
       <c r="A168" s="8" t="s">
         <v>27</v>
       </c>
@@ -6541,7 +6539,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="169" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="169" spans="1:10" ht="22.5" customHeight="1">
       <c r="A169" s="8" t="s">
         <v>27</v>
       </c>
@@ -6572,7 +6570,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="170" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="170" spans="1:10" ht="22.5" customHeight="1">
       <c r="A170" s="8" t="s">
         <v>27</v>
       </c>
@@ -6603,7 +6601,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="171" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="171" spans="1:10" ht="22.5" customHeight="1">
       <c r="A171" s="8" t="s">
         <v>27</v>
       </c>
@@ -6634,7 +6632,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="172" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="172" spans="1:10" ht="22.5" customHeight="1">
       <c r="A172" s="8" t="s">
         <v>27</v>
       </c>
@@ -6665,7 +6663,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="173" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="173" spans="1:10" ht="22.5" customHeight="1">
       <c r="A173" s="8" t="s">
         <v>27</v>
       </c>
@@ -6696,7 +6694,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="174" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="174" spans="1:10" ht="22.5" customHeight="1">
       <c r="A174" s="8" t="s">
         <v>27</v>
       </c>
@@ -6727,7 +6725,7 @@
         <v>per Patch</v>
       </c>
     </row>
-    <row r="175" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="175" spans="1:10" ht="22.5" customHeight="1">
       <c r="A175" s="8" t="s">
         <v>27</v>
       </c>
@@ -7347,7 +7345,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="195" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="195" spans="1:10" ht="22.5" customHeight="1">
       <c r="A195" s="8" t="s">
         <v>141</v>
       </c>
@@ -7378,7 +7376,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="196" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="196" spans="1:10" ht="22.5" customHeight="1">
       <c r="A196" s="8" t="s">
         <v>141</v>
       </c>
@@ -7409,7 +7407,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="197" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="197" spans="1:10" ht="22.5" customHeight="1">
       <c r="A197" s="8" t="s">
         <v>141</v>
       </c>
@@ -7440,7 +7438,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="198" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="198" spans="1:10" ht="22.5" customHeight="1">
       <c r="A198" s="8" t="s">
         <v>141</v>
       </c>
@@ -7471,7 +7469,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="199" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="199" spans="1:10" ht="22.5" customHeight="1">
       <c r="A199" s="8" t="s">
         <v>141</v>
       </c>
@@ -7502,7 +7500,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="200" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="200" spans="1:10" ht="22.5" customHeight="1">
       <c r="A200" s="8" t="s">
         <v>145</v>
       </c>
@@ -7533,7 +7531,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="201" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="201" spans="1:10" ht="22.5" customHeight="1">
       <c r="A201" s="8" t="s">
         <v>145</v>
       </c>
@@ -7564,7 +7562,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="202" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="202" spans="1:10" ht="22.5" customHeight="1">
       <c r="A202" s="8" t="s">
         <v>145</v>
       </c>
@@ -7595,7 +7593,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="203" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="203" spans="1:10" ht="22.5" customHeight="1">
       <c r="A203" s="8" t="s">
         <v>145</v>
       </c>
@@ -7626,7 +7624,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="204" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="204" spans="1:10" ht="22.5" customHeight="1">
       <c r="A204" s="8" t="s">
         <v>145</v>
       </c>
@@ -7657,7 +7655,7 @@
         <v>per Efferevescent tablet</v>
       </c>
     </row>
-    <row r="205" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="205" spans="1:10" ht="22.5" customHeight="1">
       <c r="A205" s="8" t="s">
         <v>145</v>
       </c>
@@ -7688,7 +7686,7 @@
         <v>per Efferevescent tablet</v>
       </c>
     </row>
-    <row r="206" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="206" spans="1:10" ht="22.5" customHeight="1">
       <c r="A206" s="8" t="s">
         <v>145</v>
       </c>
@@ -7719,7 +7717,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="207" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="207" spans="1:10" ht="22.5" customHeight="1">
       <c r="A207" s="8" t="s">
         <v>145</v>
       </c>
@@ -7750,7 +7748,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="208" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="208" spans="1:10" ht="22.5" customHeight="1">
       <c r="A208" s="8" t="s">
         <v>145</v>
       </c>
@@ -7781,7 +7779,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="209" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="209" spans="1:10" ht="22.5" customHeight="1">
       <c r="A209" s="8" t="s">
         <v>145</v>
       </c>
@@ -7812,7 +7810,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="210" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="210" spans="1:10" ht="22.5" customHeight="1">
       <c r="A210" s="8" t="s">
         <v>145</v>
       </c>
@@ -7843,7 +7841,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="211" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="211" spans="1:10" ht="22.5" customHeight="1">
       <c r="A211" s="8" t="s">
         <v>145</v>
       </c>
@@ -7874,7 +7872,7 @@
         <v>per Efferevescent tablet</v>
       </c>
     </row>
-    <row r="212" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="212" spans="1:10" ht="22.5" customHeight="1">
       <c r="A212" s="8" t="s">
         <v>145</v>
       </c>
@@ -7905,7 +7903,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="213" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="213" spans="1:10" ht="22.5" customHeight="1">
       <c r="A213" s="8" t="s">
         <v>145</v>
       </c>
@@ -7936,7 +7934,7 @@
         <v>per Efferevescent tablet</v>
       </c>
     </row>
-    <row r="214" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="214" spans="1:10" ht="22.5" customHeight="1">
       <c r="A214" s="8" t="s">
         <v>145</v>
       </c>
@@ -7967,7 +7965,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="215" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="215" spans="1:10" ht="22.5" customHeight="1">
       <c r="A215" s="8" t="s">
         <v>145</v>
       </c>
@@ -7998,7 +7996,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="216" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="216" spans="1:10" ht="22.5" customHeight="1">
       <c r="A216" s="8" t="s">
         <v>145</v>
       </c>
@@ -8029,7 +8027,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="217" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="217" spans="1:10" ht="22.5" customHeight="1">
       <c r="A217" s="8" t="s">
         <v>145</v>
       </c>
@@ -8060,7 +8058,7 @@
         <v>per Efferevescent tablet</v>
       </c>
     </row>
-    <row r="218" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="218" spans="1:10" ht="22.5" customHeight="1">
       <c r="A218" s="8" t="s">
         <v>145</v>
       </c>
@@ -8091,7 +8089,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="219" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="219" spans="1:10" ht="22.5" customHeight="1">
       <c r="A219" s="8" t="s">
         <v>145</v>
       </c>
@@ -8122,7 +8120,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="220" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="220" spans="1:10" ht="22.5" customHeight="1">
       <c r="A220" s="8" t="s">
         <v>145</v>
       </c>
@@ -8153,7 +8151,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="221" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="221" spans="1:10" ht="22.5" customHeight="1">
       <c r="A221" s="8" t="s">
         <v>145</v>
       </c>
@@ -8184,7 +8182,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="222" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="222" spans="1:10" ht="22.5" customHeight="1">
       <c r="A222" s="8" t="s">
         <v>145</v>
       </c>
@@ -8215,7 +8213,7 @@
         <v>per Efferevescent tablet</v>
       </c>
     </row>
-    <row r="223" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="223" spans="1:10" ht="22.5" customHeight="1">
       <c r="A223" s="8" t="s">
         <v>145</v>
       </c>
@@ -8246,7 +8244,7 @@
         <v>per Efferevescent tablet</v>
       </c>
     </row>
-    <row r="224" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="224" spans="1:10" ht="22.5" customHeight="1">
       <c r="A224" s="8" t="s">
         <v>145</v>
       </c>
@@ -8277,7 +8275,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="225" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="225" spans="1:10" ht="22.5" customHeight="1">
       <c r="A225" s="8" t="s">
         <v>155</v>
       </c>
@@ -8308,7 +8306,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="226" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="226" spans="1:10" ht="22.5" customHeight="1">
       <c r="A226" s="8" t="s">
         <v>155</v>
       </c>
@@ -8339,7 +8337,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="227" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="227" spans="1:10" ht="22.5" customHeight="1">
       <c r="A227" s="8" t="s">
         <v>155</v>
       </c>
@@ -8370,7 +8368,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="228" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="228" spans="1:10" ht="22.5" customHeight="1">
       <c r="A228" s="8" t="s">
         <v>155</v>
       </c>
@@ -8401,7 +8399,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="229" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="229" spans="1:10" ht="22.5" customHeight="1">
       <c r="A229" s="8" t="s">
         <v>155</v>
       </c>
@@ -8432,7 +8430,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="230" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="230" spans="1:10" ht="22.5" customHeight="1">
       <c r="A230" s="8" t="s">
         <v>155</v>
       </c>
@@ -8463,7 +8461,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="231" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="231" spans="1:10" ht="22.5" customHeight="1">
       <c r="A231" s="8" t="s">
         <v>155</v>
       </c>
@@ -8494,7 +8492,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="232" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="232" spans="1:10" ht="22.5" customHeight="1">
       <c r="A232" s="8" t="s">
         <v>155</v>
       </c>
@@ -8525,7 +8523,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="233" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="233" spans="1:10" ht="22.5" customHeight="1">
       <c r="A233" s="8" t="s">
         <v>155</v>
       </c>
@@ -8556,7 +8554,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="234" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="234" spans="1:10" ht="22.5" customHeight="1">
       <c r="A234" s="8" t="s">
         <v>155</v>
       </c>
@@ -8587,7 +8585,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="235" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="235" spans="1:10" ht="22.5" customHeight="1">
       <c r="A235" s="8" t="s">
         <v>155</v>
       </c>
@@ -8618,7 +8616,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="236" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="236" spans="1:10" ht="22.5" customHeight="1">
       <c r="A236" s="8" t="s">
         <v>23</v>
       </c>
@@ -8649,7 +8647,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="237" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="237" spans="1:10" ht="22.5" customHeight="1">
       <c r="A237" s="8" t="s">
         <v>23</v>
       </c>
@@ -8680,7 +8678,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="238" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="238" spans="1:10" ht="22.5" customHeight="1">
       <c r="A238" s="8" t="s">
         <v>23</v>
       </c>
@@ -8711,7 +8709,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="239" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="239" spans="1:10" ht="22.5" customHeight="1">
       <c r="A239" s="8" t="s">
         <v>23</v>
       </c>
@@ -8742,7 +8740,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="240" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="240" spans="1:10" ht="22.5" customHeight="1">
       <c r="A240" s="8" t="s">
         <v>23</v>
       </c>
@@ -8773,7 +8771,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="241" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="241" spans="1:10" ht="22.5" customHeight="1">
       <c r="A241" s="8" t="s">
         <v>23</v>
       </c>
@@ -8804,7 +8802,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="242" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="242" spans="1:10" ht="22.5" customHeight="1">
       <c r="A242" s="8" t="s">
         <v>23</v>
       </c>
@@ -8835,7 +8833,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="243" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="243" spans="1:10" ht="22.5" customHeight="1">
       <c r="A243" s="8" t="s">
         <v>23</v>
       </c>
@@ -8866,7 +8864,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="244" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="244" spans="1:10" ht="22.5" customHeight="1">
       <c r="A244" s="8" t="s">
         <v>27</v>
       </c>
@@ -8897,7 +8895,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="245" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="245" spans="1:10" ht="22.5" customHeight="1">
       <c r="A245" s="8" t="s">
         <v>27</v>
       </c>
@@ -8928,7 +8926,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="246" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="246" spans="1:10" ht="22.5" customHeight="1">
       <c r="A246" s="8" t="s">
         <v>27</v>
       </c>
@@ -8959,7 +8957,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="247" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="247" spans="1:10" ht="22.5" customHeight="1">
       <c r="A247" s="8" t="s">
         <v>27</v>
       </c>
@@ -8990,7 +8988,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="248" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="248" spans="1:10" ht="22.5" customHeight="1">
       <c r="A248" s="8" t="s">
         <v>27</v>
       </c>
@@ -9021,7 +9019,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="249" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="249" spans="1:10" ht="22.5" customHeight="1">
       <c r="A249" s="8" t="s">
         <v>27</v>
       </c>
@@ -9052,7 +9050,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="250" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="250" spans="1:10" ht="22.5" customHeight="1">
       <c r="A250" s="8" t="s">
         <v>27</v>
       </c>
@@ -9083,7 +9081,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="251" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="251" spans="1:10" ht="22.5" customHeight="1">
       <c r="A251" s="8" t="s">
         <v>27</v>
       </c>
@@ -9114,7 +9112,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="252" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="252" spans="1:10" ht="22.5" customHeight="1">
       <c r="A252" s="8" t="s">
         <v>27</v>
       </c>
@@ -9145,7 +9143,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="253" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="253" spans="1:10" ht="22.5" customHeight="1">
       <c r="A253" s="8" t="s">
         <v>27</v>
       </c>
@@ -9176,7 +9174,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="254" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="254" spans="1:10" ht="22.5" customHeight="1">
       <c r="A254" s="8" t="s">
         <v>27</v>
       </c>
@@ -9207,7 +9205,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="255" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="255" spans="1:10" ht="22.5" customHeight="1">
       <c r="A255" s="8" t="s">
         <v>27</v>
       </c>
@@ -9238,7 +9236,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="256" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="256" spans="1:10" ht="22.5" customHeight="1">
       <c r="A256" s="8" t="s">
         <v>27</v>
       </c>
@@ -9269,7 +9267,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="257" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="257" spans="1:10" ht="22.5" customHeight="1">
       <c r="A257" s="8" t="s">
         <v>27</v>
       </c>
@@ -9300,7 +9298,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="258" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="258" spans="1:10" ht="22.5" customHeight="1">
       <c r="A258" s="8" t="s">
         <v>27</v>
       </c>
@@ -9331,7 +9329,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="259" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="259" spans="1:10" ht="22.5" customHeight="1">
       <c r="A259" s="8" t="s">
         <v>27</v>
       </c>
@@ -9362,7 +9360,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="260" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="260" spans="1:10" ht="22.5" customHeight="1">
       <c r="A260" s="8" t="s">
         <v>27</v>
       </c>
@@ -9393,7 +9391,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="261" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="261" spans="1:10" ht="22.5" customHeight="1">
       <c r="A261" s="8" t="s">
         <v>27</v>
       </c>
@@ -9424,7 +9422,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="262" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="262" spans="1:10" ht="22.5" customHeight="1">
       <c r="A262" s="8" t="s">
         <v>27</v>
       </c>
@@ -9455,7 +9453,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="263" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="263" spans="1:10" ht="22.5" customHeight="1">
       <c r="A263" s="8" t="s">
         <v>27</v>
       </c>
@@ -9486,7 +9484,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="264" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="264" spans="1:10" ht="22.5" customHeight="1">
       <c r="A264" s="8" t="s">
         <v>175</v>
       </c>
@@ -9517,7 +9515,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="265" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="265" spans="1:10" ht="22.5" customHeight="1">
       <c r="A265" s="8" t="s">
         <v>175</v>
       </c>
@@ -9548,7 +9546,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="266" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="266" spans="1:10" ht="22.5" customHeight="1">
       <c r="A266" s="8" t="s">
         <v>175</v>
       </c>
@@ -9579,7 +9577,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="267" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="267" spans="1:10" ht="22.5" customHeight="1">
       <c r="A267" s="8" t="s">
         <v>175</v>
       </c>
@@ -9610,7 +9608,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="268" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="268" spans="1:10" ht="22.5" customHeight="1">
       <c r="A268" s="8" t="s">
         <v>175</v>
       </c>
@@ -9641,7 +9639,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="269" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="269" spans="1:10" ht="22.5" customHeight="1">
       <c r="A269" s="8" t="s">
         <v>175</v>
       </c>
@@ -9672,7 +9670,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="270" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="270" spans="1:10" ht="22.5" customHeight="1">
       <c r="A270" s="8" t="s">
         <v>175</v>
       </c>
@@ -9703,7 +9701,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="271" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="271" spans="1:10" ht="22.5" customHeight="1">
       <c r="A271" s="8" t="s">
         <v>35</v>
       </c>
@@ -9734,7 +9732,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="272" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="272" spans="1:10" ht="22.5" customHeight="1">
       <c r="A272" s="8" t="s">
         <v>82</v>
       </c>
@@ -9765,7 +9763,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="273" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="273" spans="1:10" ht="22.5" customHeight="1">
       <c r="A273" s="8" t="s">
         <v>50</v>
       </c>
@@ -9796,7 +9794,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="274" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="274" spans="1:10" ht="22.5" customHeight="1">
       <c r="A274" s="8" t="s">
         <v>50</v>
       </c>
@@ -9827,7 +9825,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="275" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="275" spans="1:10" ht="22.5" customHeight="1">
       <c r="A275" s="8" t="s">
         <v>50</v>
       </c>
@@ -9858,7 +9856,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="276" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="276" spans="1:10" ht="22.5" customHeight="1">
       <c r="A276" s="8" t="s">
         <v>50</v>
       </c>
@@ -9889,7 +9887,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="277" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="277" spans="1:10" ht="22.5" customHeight="1">
       <c r="A277" s="8" t="s">
         <v>50</v>
       </c>
@@ -9920,7 +9918,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="278" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="278" spans="1:10" ht="22.5" customHeight="1">
       <c r="A278" s="8" t="s">
         <v>50</v>
       </c>
@@ -9951,7 +9949,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="279" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="279" spans="1:10" ht="22.5" customHeight="1">
       <c r="A279" s="8" t="s">
         <v>50</v>
       </c>
@@ -9982,7 +9980,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="280" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="280" spans="1:10" ht="22.5" customHeight="1">
       <c r="A280" s="8" t="s">
         <v>50</v>
       </c>
@@ -10013,7 +10011,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="281" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="281" spans="1:10" ht="22.5" customHeight="1">
       <c r="A281" s="8" t="s">
         <v>50</v>
       </c>
@@ -10044,7 +10042,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="282" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="282" spans="1:10" ht="22.5" customHeight="1">
       <c r="A282" s="8" t="s">
         <v>50</v>
       </c>
@@ -10075,7 +10073,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="283" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="283" spans="1:10" ht="22.5" customHeight="1">
       <c r="A283" s="8" t="s">
         <v>50</v>
       </c>
@@ -10106,7 +10104,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="284" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="284" spans="1:10" ht="22.5" customHeight="1">
       <c r="A284" s="8" t="s">
         <v>50</v>
       </c>
@@ -10137,7 +10135,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="285" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="285" spans="1:10" ht="22.5" customHeight="1">
       <c r="A285" s="8" t="s">
         <v>50</v>
       </c>
@@ -10168,7 +10166,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="286" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="286" spans="1:10" ht="22.5" customHeight="1">
       <c r="A286" s="8" t="s">
         <v>50</v>
       </c>
@@ -10199,7 +10197,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="287" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="287" spans="1:10" ht="22.5" customHeight="1">
       <c r="A287" s="8" t="s">
         <v>66</v>
       </c>
@@ -10230,7 +10228,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="288" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="288" spans="1:10" ht="22.5" customHeight="1">
       <c r="A288" s="8" t="s">
         <v>66</v>
       </c>
@@ -10261,7 +10259,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="289" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="289" spans="1:10" ht="22.5" customHeight="1">
       <c r="A289" s="8" t="s">
         <v>66</v>
       </c>
@@ -10292,7 +10290,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="290" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="290" spans="1:10" ht="22.5" customHeight="1">
       <c r="A290" s="8" t="s">
         <v>66</v>
       </c>
@@ -10323,7 +10321,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="291" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="291" spans="1:10" ht="22.5" customHeight="1">
       <c r="A291" s="8" t="s">
         <v>66</v>
       </c>
@@ -10354,7 +10352,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="292" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="292" spans="1:10" ht="22.5" customHeight="1">
       <c r="A292" s="8" t="s">
         <v>66</v>
       </c>
@@ -10385,7 +10383,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="293" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="293" spans="1:10" ht="22.5" customHeight="1">
       <c r="A293" s="8" t="s">
         <v>66</v>
       </c>
@@ -10416,7 +10414,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="294" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="294" spans="1:10" ht="22.5" customHeight="1">
       <c r="A294" s="8" t="s">
         <v>66</v>
       </c>
@@ -10447,7 +10445,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="295" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="295" spans="1:10" ht="22.5" customHeight="1">
       <c r="A295" s="8" t="s">
         <v>66</v>
       </c>
@@ -10478,7 +10476,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="296" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="296" spans="1:10" ht="22.5" customHeight="1">
       <c r="A296" s="8" t="s">
         <v>66</v>
       </c>
@@ -10509,7 +10507,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="297" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="297" spans="1:10" ht="22.5" customHeight="1">
       <c r="A297" s="8" t="s">
         <v>66</v>
       </c>
@@ -10540,7 +10538,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="298" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="298" spans="1:10" ht="22.5" customHeight="1">
       <c r="A298" s="8" t="s">
         <v>66</v>
       </c>
@@ -10571,7 +10569,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="299" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="299" spans="1:10" ht="22.5" customHeight="1">
       <c r="A299" s="8" t="s">
         <v>66</v>
       </c>
@@ -10602,7 +10600,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="300" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="300" spans="1:10" ht="22.5" customHeight="1">
       <c r="A300" s="8" t="s">
         <v>66</v>
       </c>
@@ -10633,7 +10631,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="301" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="301" spans="1:10" ht="22.5" customHeight="1">
       <c r="A301" s="8" t="s">
         <v>66</v>
       </c>
@@ -10664,7 +10662,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="302" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="302" spans="1:10" ht="22.5" customHeight="1">
       <c r="A302" s="8" t="s">
         <v>66</v>
       </c>
@@ -10695,7 +10693,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="303" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="303" spans="1:10" ht="22.5" customHeight="1">
       <c r="A303" s="8" t="s">
         <v>66</v>
       </c>
@@ -10726,7 +10724,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="304" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="304" spans="1:10" ht="22.5" customHeight="1">
       <c r="A304" s="8" t="s">
         <v>66</v>
       </c>
@@ -10757,7 +10755,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="305" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="305" spans="1:10" ht="22.5" customHeight="1">
       <c r="A305" s="8" t="s">
         <v>66</v>
       </c>
@@ -10788,7 +10786,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="306" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="306" spans="1:10" ht="22.5" customHeight="1">
       <c r="A306" s="8" t="s">
         <v>66</v>
       </c>
@@ -10819,7 +10817,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="307" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="307" spans="1:10" ht="22.5" customHeight="1">
       <c r="A307" s="8" t="s">
         <v>66</v>
       </c>
@@ -10850,7 +10848,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="308" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="308" spans="1:10" ht="22.5" customHeight="1">
       <c r="A308" s="8" t="s">
         <v>66</v>
       </c>
@@ -10881,7 +10879,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="309" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="309" spans="1:10" ht="22.5" customHeight="1">
       <c r="A309" s="8" t="s">
         <v>66</v>
       </c>
@@ -10912,7 +10910,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="310" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="310" spans="1:10" ht="22.5" customHeight="1">
       <c r="A310" s="8" t="s">
         <v>66</v>
       </c>
@@ -10943,7 +10941,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="311" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="311" spans="1:10" ht="22.5" customHeight="1">
       <c r="A311" s="8" t="s">
         <v>66</v>
       </c>
@@ -10974,7 +10972,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="312" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="312" spans="1:10" ht="22.5" customHeight="1">
       <c r="A312" s="8" t="s">
         <v>66</v>
       </c>
@@ -11005,7 +11003,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="313" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="313" spans="1:10" ht="22.5" customHeight="1">
       <c r="A313" s="8" t="s">
         <v>66</v>
       </c>
@@ -11036,7 +11034,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="314" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="314" spans="1:10" ht="22.5" customHeight="1">
       <c r="A314" s="8" t="s">
         <v>66</v>
       </c>
@@ -11067,7 +11065,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="315" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="315" spans="1:10" ht="22.5" customHeight="1">
       <c r="A315" s="8" t="s">
         <v>66</v>
       </c>
@@ -11098,7 +11096,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="316" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="316" spans="1:10" ht="22.5" customHeight="1">
       <c r="A316" s="8" t="s">
         <v>66</v>
       </c>
@@ -11129,7 +11127,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="317" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="317" spans="1:10" ht="22.5" customHeight="1">
       <c r="A317" s="8" t="s">
         <v>66</v>
       </c>
@@ -11160,7 +11158,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="318" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="318" spans="1:10" ht="22.5" customHeight="1">
       <c r="A318" s="8" t="s">
         <v>66</v>
       </c>
@@ -11191,7 +11189,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="319" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="319" spans="1:10" ht="22.5" customHeight="1">
       <c r="A319" s="8" t="s">
         <v>66</v>
       </c>
@@ -11222,7 +11220,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="320" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="320" spans="1:10" ht="22.5" customHeight="1">
       <c r="A320" s="8" t="s">
         <v>66</v>
       </c>
@@ -11253,7 +11251,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="321" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="321" spans="1:10" ht="22.5" customHeight="1">
       <c r="A321" s="8" t="s">
         <v>66</v>
       </c>
@@ -11284,7 +11282,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="322" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="322" spans="1:10" ht="22.5" customHeight="1">
       <c r="A322" s="8" t="s">
         <v>66</v>
       </c>
@@ -11315,7 +11313,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="323" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="323" spans="1:10" ht="22.5" customHeight="1">
       <c r="A323" s="8" t="s">
         <v>66</v>
       </c>
@@ -11346,7 +11344,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="324" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="324" spans="1:10" ht="22.5" customHeight="1">
       <c r="A324" s="8" t="s">
         <v>66</v>
       </c>
@@ -11377,7 +11375,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="325" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="325" spans="1:10" ht="22.5" customHeight="1">
       <c r="A325" s="8" t="s">
         <v>66</v>
       </c>
@@ -11408,7 +11406,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="326" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="326" spans="1:10" ht="22.5" customHeight="1">
       <c r="A326" s="8" t="s">
         <v>69</v>
       </c>
@@ -11439,7 +11437,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="327" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="327" spans="1:10" ht="22.5" customHeight="1">
       <c r="A327" s="8" t="s">
         <v>88</v>
       </c>
@@ -11470,7 +11468,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="328" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="328" spans="1:10" ht="22.5" customHeight="1">
       <c r="A328" s="8" t="s">
         <v>88</v>
       </c>
@@ -11501,7 +11499,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="329" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="329" spans="1:10" ht="22.5" customHeight="1">
       <c r="A329" s="8" t="s">
         <v>88</v>
       </c>
@@ -11532,7 +11530,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="330" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="330" spans="1:10" ht="22.5" customHeight="1">
       <c r="A330" s="8" t="s">
         <v>88</v>
       </c>
@@ -11563,7 +11561,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="331" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="331" spans="1:10" ht="22.5" customHeight="1">
       <c r="A331" s="8" t="s">
         <v>88</v>
       </c>
@@ -11594,7 +11592,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="332" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="332" spans="1:10" ht="22.5" customHeight="1">
       <c r="A332" s="8" t="s">
         <v>88</v>
       </c>
@@ -11625,7 +11623,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="333" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="333" spans="1:10" ht="22.5" customHeight="1">
       <c r="A333" s="8" t="s">
         <v>88</v>
       </c>
@@ -11656,7 +11654,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="334" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="334" spans="1:10" ht="22.5" customHeight="1">
       <c r="A334" s="8" t="s">
         <v>88</v>
       </c>
@@ -11687,7 +11685,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="335" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="335" spans="1:10" ht="22.5" customHeight="1">
       <c r="A335" s="8" t="s">
         <v>88</v>
       </c>
@@ -11718,7 +11716,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="336" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="336" spans="1:10" ht="22.5" customHeight="1">
       <c r="A336" s="8" t="s">
         <v>88</v>
       </c>
@@ -11749,7 +11747,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="337" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="337" spans="1:10" ht="22.5" customHeight="1">
       <c r="A337" s="8" t="s">
         <v>71</v>
       </c>
@@ -11780,7 +11778,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="338" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="338" spans="1:10" ht="22.5" customHeight="1">
       <c r="A338" s="8" t="s">
         <v>71</v>
       </c>
@@ -11811,7 +11809,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="339" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="339" spans="1:10" ht="22.5" customHeight="1">
       <c r="A339" s="8" t="s">
         <v>71</v>
       </c>
@@ -11842,7 +11840,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="340" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="340" spans="1:10" ht="22.5" customHeight="1">
       <c r="A340" s="8" t="s">
         <v>71</v>
       </c>
@@ -11873,7 +11871,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="341" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="341" spans="1:10" ht="22.5" customHeight="1">
       <c r="A341" s="8" t="s">
         <v>71</v>
       </c>
@@ -11904,7 +11902,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="342" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="342" spans="1:10" ht="22.5" customHeight="1">
       <c r="A342" s="8" t="s">
         <v>71</v>
       </c>
@@ -11935,7 +11933,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="343" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="343" spans="1:10" ht="22.5" customHeight="1">
       <c r="A343" s="8" t="s">
         <v>71</v>
       </c>
@@ -11966,7 +11964,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="344" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="344" spans="1:10" ht="22.5" customHeight="1">
       <c r="A344" s="8" t="s">
         <v>71</v>
       </c>
@@ -11997,7 +11995,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="345" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="345" spans="1:10" ht="22.5" customHeight="1">
       <c r="A345" s="8" t="s">
         <v>71</v>
       </c>
@@ -12028,7 +12026,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="346" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="346" spans="1:10" ht="22.5" customHeight="1">
       <c r="A346" s="8" t="s">
         <v>71</v>
       </c>
@@ -12059,7 +12057,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="347" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="347" spans="1:10" ht="22.5" customHeight="1">
       <c r="A347" s="8" t="s">
         <v>71</v>
       </c>
@@ -12090,7 +12088,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="348" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="348" spans="1:10" ht="22.5" customHeight="1">
       <c r="A348" s="8" t="s">
         <v>71</v>
       </c>
@@ -12121,7 +12119,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="349" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="349" spans="1:10" ht="22.5" customHeight="1">
       <c r="A349" s="8" t="s">
         <v>71</v>
       </c>
@@ -12152,7 +12150,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="350" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="350" spans="1:10" ht="22.5" customHeight="1">
       <c r="A350" s="8" t="s">
         <v>71</v>
       </c>
@@ -12183,7 +12181,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="351" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="351" spans="1:10" ht="22.5" customHeight="1">
       <c r="A351" s="8" t="s">
         <v>71</v>
       </c>
@@ -12214,7 +12212,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="352" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="352" spans="1:10" ht="22.5" customHeight="1">
       <c r="A352" s="8" t="s">
         <v>71</v>
       </c>
@@ -12245,7 +12243,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="353" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="353" spans="1:10" ht="22.5" customHeight="1">
       <c r="A353" s="8" t="s">
         <v>71</v>
       </c>
@@ -12276,7 +12274,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="354" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="354" spans="1:10" ht="22.5" customHeight="1">
       <c r="A354" s="8" t="s">
         <v>71</v>
       </c>
@@ -12307,7 +12305,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="355" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="355" spans="1:10" ht="22.5" customHeight="1">
       <c r="A355" s="8" t="s">
         <v>71</v>
       </c>
@@ -12338,7 +12336,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="356" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="356" spans="1:10" ht="22.5" customHeight="1">
       <c r="A356" s="8" t="s">
         <v>71</v>
       </c>
@@ -12369,7 +12367,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="357" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="357" spans="1:10" ht="22.5" customHeight="1">
       <c r="A357" s="8" t="s">
         <v>71</v>
       </c>
@@ -12400,7 +12398,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="358" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="358" spans="1:10" ht="22.5" customHeight="1">
       <c r="A358" s="8" t="s">
         <v>71</v>
       </c>
@@ -12431,7 +12429,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="359" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="359" spans="1:10" ht="22.5" customHeight="1">
       <c r="A359" s="8" t="s">
         <v>71</v>
       </c>
@@ -12462,7 +12460,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="360" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="360" spans="1:10" ht="22.5" customHeight="1">
       <c r="A360" s="8" t="s">
         <v>71</v>
       </c>
@@ -12493,7 +12491,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="361" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="361" spans="1:10" ht="22.5" customHeight="1">
       <c r="A361" s="8" t="s">
         <v>71</v>
       </c>
@@ -12524,7 +12522,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="362" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="362" spans="1:10" ht="22.5" customHeight="1">
       <c r="A362" s="8" t="s">
         <v>71</v>
       </c>
@@ -12555,7 +12553,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="363" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="363" spans="1:10" ht="22.5" customHeight="1">
       <c r="A363" s="8" t="s">
         <v>71</v>
       </c>
@@ -12586,7 +12584,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="364" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="364" spans="1:10" ht="22.5" customHeight="1">
       <c r="A364" s="8" t="s">
         <v>71</v>
       </c>
@@ -12617,7 +12615,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="365" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="365" spans="1:10" ht="22.5" customHeight="1">
       <c r="A365" s="8" t="s">
         <v>71</v>
       </c>
@@ -12648,7 +12646,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="366" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="366" spans="1:10" ht="22.5" customHeight="1">
       <c r="A366" s="8" t="s">
         <v>71</v>
       </c>
@@ -12679,7 +12677,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="367" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="367" spans="1:10" ht="22.5" customHeight="1">
       <c r="A367" s="8" t="s">
         <v>71</v>
       </c>
@@ -12710,7 +12708,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="368" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="368" spans="1:10" ht="22.5" customHeight="1">
       <c r="A368" s="8" t="s">
         <v>71</v>
       </c>
@@ -12741,7 +12739,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="369" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="369" spans="1:10" ht="22.5" customHeight="1">
       <c r="A369" s="8" t="s">
         <v>71</v>
       </c>
@@ -12772,7 +12770,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="370" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="370" spans="1:10" ht="22.5" customHeight="1">
       <c r="A370" s="8" t="s">
         <v>71</v>
       </c>
@@ -12803,7 +12801,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="371" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="371" spans="1:10" ht="22.5" customHeight="1">
       <c r="A371" s="8" t="s">
         <v>71</v>
       </c>
@@ -12834,7 +12832,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="372" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="372" spans="1:10" ht="22.5" customHeight="1">
       <c r="A372" s="8" t="s">
         <v>71</v>
       </c>
@@ -12865,7 +12863,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="373" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="373" spans="1:10" ht="22.5" customHeight="1">
       <c r="A373" s="8" t="s">
         <v>71</v>
       </c>
@@ -12896,7 +12894,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="374" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="374" spans="1:10" ht="22.5" customHeight="1">
       <c r="A374" s="8" t="s">
         <v>71</v>
       </c>
@@ -12927,7 +12925,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="375" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="375" spans="1:10" ht="22.5" customHeight="1">
       <c r="A375" s="8" t="s">
         <v>71</v>
       </c>
@@ -12958,7 +12956,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="376" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="376" spans="1:10" ht="22.5" customHeight="1">
       <c r="A376" s="8" t="s">
         <v>71</v>
       </c>
@@ -12989,7 +12987,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="377" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="377" spans="1:10" ht="22.5" customHeight="1">
       <c r="A377" s="8" t="s">
         <v>71</v>
       </c>
@@ -13020,7 +13018,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="378" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="378" spans="1:10" ht="22.5" customHeight="1">
       <c r="A378" s="8" t="s">
         <v>71</v>
       </c>
@@ -13051,7 +13049,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="379" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="379" spans="1:10" ht="22.5" customHeight="1">
       <c r="A379" s="8" t="s">
         <v>71</v>
       </c>
@@ -13082,7 +13080,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="380" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="380" spans="1:10" ht="22.5" customHeight="1">
       <c r="A380" s="8" t="s">
         <v>71</v>
       </c>
@@ -13113,7 +13111,7 @@
         <v>per Tablet</v>
       </c>
     </row>
-    <row r="381" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="381" spans="1:10" ht="22.5" customHeight="1">
       <c r="A381" s="3"/>
       <c r="B381" s="4"/>
       <c r="C381" s="3"/>
@@ -13124,7 +13122,7 @@
       <c r="H381" s="4"/>
       <c r="I381" s="4"/>
     </row>
-    <row r="382" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="382" spans="1:10" ht="22.5" customHeight="1">
       <c r="A382" s="3"/>
       <c r="B382" s="4"/>
       <c r="C382" s="3"/>
@@ -13135,7 +13133,7 @@
       <c r="H382" s="4"/>
       <c r="I382" s="4"/>
     </row>
-    <row r="383" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="383" spans="1:10" ht="22.5" customHeight="1">
       <c r="A383" s="3"/>
       <c r="B383" s="4"/>
       <c r="C383" s="3"/>
@@ -13146,7 +13144,7 @@
       <c r="H383" s="4"/>
       <c r="I383" s="4"/>
     </row>
-    <row r="384" spans="1:10" ht="22.5" hidden="1" customHeight="1">
+    <row r="384" spans="1:10" ht="22.5" customHeight="1">
       <c r="A384" s="3"/>
       <c r="B384" s="4"/>
       <c r="C384" s="3"/>
@@ -13157,7 +13155,7 @@
       <c r="H384" s="4"/>
       <c r="I384" s="4"/>
     </row>
-    <row r="385" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="385" spans="1:9" ht="22.5" customHeight="1">
       <c r="A385" s="3"/>
       <c r="B385" s="4"/>
       <c r="C385" s="3"/>
@@ -13168,7 +13166,7 @@
       <c r="H385" s="4"/>
       <c r="I385" s="4"/>
     </row>
-    <row r="386" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="386" spans="1:9" ht="22.5" customHeight="1">
       <c r="A386" s="3"/>
       <c r="B386" s="4"/>
       <c r="C386" s="3"/>
@@ -13179,7 +13177,7 @@
       <c r="H386" s="4"/>
       <c r="I386" s="4"/>
     </row>
-    <row r="387" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="387" spans="1:9" ht="22.5" customHeight="1">
       <c r="A387" s="3"/>
       <c r="B387" s="4"/>
       <c r="C387" s="3"/>
@@ -13190,7 +13188,7 @@
       <c r="H387" s="4"/>
       <c r="I387" s="4"/>
     </row>
-    <row r="388" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="388" spans="1:9" ht="22.5" customHeight="1">
       <c r="A388" s="3"/>
       <c r="B388" s="4"/>
       <c r="C388" s="3"/>
@@ -13201,7 +13199,7 @@
       <c r="H388" s="4"/>
       <c r="I388" s="4"/>
     </row>
-    <row r="389" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="389" spans="1:9" ht="22.5" customHeight="1">
       <c r="A389" s="3"/>
       <c r="B389" s="4"/>
       <c r="C389" s="3"/>
@@ -13212,7 +13210,7 @@
       <c r="H389" s="4"/>
       <c r="I389" s="4"/>
     </row>
-    <row r="390" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="390" spans="1:9" ht="22.5" customHeight="1">
       <c r="A390" s="3"/>
       <c r="B390" s="4"/>
       <c r="C390" s="3"/>
@@ -13223,7 +13221,7 @@
       <c r="H390" s="4"/>
       <c r="I390" s="4"/>
     </row>
-    <row r="391" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="391" spans="1:9" ht="22.5" customHeight="1">
       <c r="A391" s="3"/>
       <c r="B391" s="4"/>
       <c r="C391" s="3"/>
@@ -13234,7 +13232,7 @@
       <c r="H391" s="4"/>
       <c r="I391" s="4"/>
     </row>
-    <row r="392" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="392" spans="1:9" ht="22.5" customHeight="1">
       <c r="A392" s="3"/>
       <c r="B392" s="4"/>
       <c r="C392" s="3"/>
@@ -13245,7 +13243,7 @@
       <c r="H392" s="4"/>
       <c r="I392" s="4"/>
     </row>
-    <row r="393" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="393" spans="1:9" ht="22.5" customHeight="1">
       <c r="A393" s="3"/>
       <c r="B393" s="4"/>
       <c r="C393" s="3"/>
@@ -13256,7 +13254,7 @@
       <c r="H393" s="4"/>
       <c r="I393" s="4"/>
     </row>
-    <row r="394" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="394" spans="1:9" ht="22.5" customHeight="1">
       <c r="A394" s="3"/>
       <c r="B394" s="4"/>
       <c r="C394" s="3"/>
@@ -13267,7 +13265,7 @@
       <c r="H394" s="4"/>
       <c r="I394" s="4"/>
     </row>
-    <row r="395" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="395" spans="1:9" ht="22.5" customHeight="1">
       <c r="A395" s="3"/>
       <c r="B395" s="4"/>
       <c r="C395" s="3"/>
@@ -13278,7 +13276,7 @@
       <c r="H395" s="4"/>
       <c r="I395" s="4"/>
     </row>
-    <row r="396" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="396" spans="1:9" ht="22.5" customHeight="1">
       <c r="A396" s="3"/>
       <c r="B396" s="4"/>
       <c r="C396" s="3"/>
@@ -13289,7 +13287,7 @@
       <c r="H396" s="4"/>
       <c r="I396" s="4"/>
     </row>
-    <row r="397" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="397" spans="1:9" ht="22.5" customHeight="1">
       <c r="A397" s="3"/>
       <c r="B397" s="4"/>
       <c r="C397" s="3"/>
@@ -13300,7 +13298,7 @@
       <c r="H397" s="4"/>
       <c r="I397" s="4"/>
     </row>
-    <row r="398" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="398" spans="1:9" ht="22.5" customHeight="1">
       <c r="A398" s="3"/>
       <c r="B398" s="4"/>
       <c r="C398" s="3"/>
@@ -13311,7 +13309,7 @@
       <c r="H398" s="4"/>
       <c r="I398" s="4"/>
     </row>
-    <row r="399" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="399" spans="1:9" ht="22.5" customHeight="1">
       <c r="A399" s="3"/>
       <c r="B399" s="4"/>
       <c r="C399" s="3"/>
@@ -13322,7 +13320,7 @@
       <c r="H399" s="4"/>
       <c r="I399" s="4"/>
     </row>
-    <row r="400" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="400" spans="1:9" ht="22.5" customHeight="1">
       <c r="A400" s="3"/>
       <c r="B400" s="4"/>
       <c r="C400" s="3"/>
@@ -13333,7 +13331,7 @@
       <c r="H400" s="4"/>
       <c r="I400" s="4"/>
     </row>
-    <row r="401" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="401" spans="1:9" ht="22.5" customHeight="1">
       <c r="A401" s="3"/>
       <c r="B401" s="4"/>
       <c r="C401" s="3"/>
@@ -13344,7 +13342,7 @@
       <c r="H401" s="4"/>
       <c r="I401" s="4"/>
     </row>
-    <row r="402" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="402" spans="1:9" ht="22.5" customHeight="1">
       <c r="A402" s="3"/>
       <c r="B402" s="4"/>
       <c r="C402" s="3"/>
@@ -13355,7 +13353,7 @@
       <c r="H402" s="4"/>
       <c r="I402" s="4"/>
     </row>
-    <row r="403" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="403" spans="1:9" ht="22.5" customHeight="1">
       <c r="A403" s="3"/>
       <c r="B403" s="4"/>
       <c r="C403" s="3"/>
@@ -13366,7 +13364,7 @@
       <c r="H403" s="4"/>
       <c r="I403" s="4"/>
     </row>
-    <row r="404" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="404" spans="1:9" ht="22.5" customHeight="1">
       <c r="A404" s="3"/>
       <c r="B404" s="4"/>
       <c r="C404" s="3"/>
@@ -13377,7 +13375,7 @@
       <c r="H404" s="4"/>
       <c r="I404" s="4"/>
     </row>
-    <row r="405" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="405" spans="1:9" ht="22.5" customHeight="1">
       <c r="A405" s="3"/>
       <c r="B405" s="4"/>
       <c r="C405" s="3"/>
@@ -13388,7 +13386,7 @@
       <c r="H405" s="4"/>
       <c r="I405" s="4"/>
     </row>
-    <row r="406" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="406" spans="1:9" ht="22.5" customHeight="1">
       <c r="A406" s="3"/>
       <c r="B406" s="4"/>
       <c r="C406" s="3"/>
@@ -13399,7 +13397,7 @@
       <c r="H406" s="4"/>
       <c r="I406" s="4"/>
     </row>
-    <row r="407" spans="1:9" ht="22.5" hidden="1" customHeight="1">
+    <row r="407" spans="1:9" ht="22.5" customHeight="1">
       <c r="A407" s="3"/>
       <c r="B407" s="4"/>
       <c r="C407" s="3"/>
@@ -13411,18 +13409,6 @@
       <c r="I407" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B407" xr:uid="{537DEBE9-B305-49C6-BA8B-E5C9DA8CC8BE}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Buprenorphine"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Tablet"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A200:J224">
     <sortCondition ref="C2:C407"/>
   </sortState>

</xml_diff>